<commit_message>
Update AIP fuel price files and documentation
</commit_message>
<xml_diff>
--- a/data/AIP_fuel_prices_formatted.xlsx
+++ b/data/AIP_fuel_prices_formatted.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ULP" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Diesel'!$A$1:$K$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ULP'!$A$1:$K$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Diesel'!$A$1:$I$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ULP'!$A$1:$I$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="d mmm yyyy"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,9 +39,6 @@
     <font>
       <color rgb="002F7E8E"/>
       <u val="single"/>
-    </font>
-    <font>
-      <color rgb="00000000"/>
     </font>
   </fonts>
   <fills count="2">
@@ -84,16 +81,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -473,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -485,8 +479,6 @@
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -535,1739 +527,1621 @@
           <t>National Average</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>Excise Cut (1 Apr)</t>
-        </is>
-      </c>
-      <c r="K1" s="4" t="inlineStr">
-        <is>
-          <t>Fuel Price Lock (20 Apr)</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n">
+      <c r="A2" s="4" t="n">
         <v>45809</v>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>1 Jun</t>
         </is>
       </c>
-      <c r="C2" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D2" s="8" t="n">
+      <c r="C2" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D2" s="7" t="n">
         <v>181.1</v>
       </c>
-      <c r="E2" s="8" t="n">
+      <c r="E2" s="7" t="n">
         <v>238.7</v>
       </c>
-      <c r="F2" s="8" t="n">
+      <c r="F2" s="7" t="n">
         <v>203.8</v>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="G2" s="7" t="n">
         <v>175.5</v>
       </c>
-      <c r="H2" s="8" t="n">
+      <c r="H2" s="7" t="n">
         <v>180.1</v>
       </c>
-      <c r="I2" s="8" t="n">
+      <c r="I2" s="7" t="n">
         <v>178</v>
       </c>
-      <c r="J2" s="8" t="n">
-        <v>300</v>
-      </c>
-      <c r="K2" s="8" t="n">
-        <v>300</v>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="4" t="n">
         <v>45816</v>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>8 Jun</t>
         </is>
       </c>
-      <c r="C3" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D3" s="8" t="n">
+      <c r="C3" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D3" s="7" t="n">
         <v>181</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="7" t="n">
         <v>238.8</v>
       </c>
-      <c r="F3" s="8" t="n">
+      <c r="F3" s="7" t="n">
         <v>203.7</v>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="G3" s="7" t="n">
         <v>175</v>
       </c>
-      <c r="H3" s="8" t="n">
+      <c r="H3" s="7" t="n">
         <v>179.7</v>
       </c>
-      <c r="I3" s="8" t="n">
+      <c r="I3" s="7" t="n">
         <v>177.6</v>
       </c>
-      <c r="J3" s="6" t="inlineStr"/>
-      <c r="K3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="4" t="n">
         <v>45823</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>15 Jun</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D4" s="8" t="n">
+      <c r="C4" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D4" s="7" t="n">
         <v>181.1</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="7" t="n">
         <v>238.4</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="7" t="n">
         <v>203.6</v>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="G4" s="7" t="n">
         <v>175</v>
       </c>
-      <c r="H4" s="8" t="n">
+      <c r="H4" s="7" t="n">
         <v>179.5</v>
       </c>
-      <c r="I4" s="8" t="n">
+      <c r="I4" s="7" t="n">
         <v>177.5</v>
       </c>
-      <c r="J4" s="6" t="inlineStr"/>
-      <c r="K4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="4" t="n">
         <v>45830</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>22 Jun</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D5" s="8" t="n">
+      <c r="C5" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D5" s="7" t="n">
         <v>182</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="7" t="n">
         <v>238.7</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="7" t="n">
         <v>204.3</v>
       </c>
-      <c r="G5" s="8" t="n">
+      <c r="G5" s="7" t="n">
         <v>177.8</v>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="H5" s="7" t="n">
         <v>181.6</v>
       </c>
-      <c r="I5" s="8" t="n">
+      <c r="I5" s="7" t="n">
         <v>179.9</v>
       </c>
-      <c r="J5" s="6" t="inlineStr"/>
-      <c r="K5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="4" t="n">
         <v>45837</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>29 Jun</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D6" s="8" t="n">
+      <c r="C6" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D6" s="7" t="n">
         <v>184.7</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="7" t="n">
         <v>239.8</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="7" t="n">
         <v>206.4</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="7" t="n">
         <v>183.3</v>
       </c>
-      <c r="H6" s="8" t="n">
+      <c r="H6" s="7" t="n">
         <v>186.7</v>
       </c>
-      <c r="I6" s="8" t="n">
+      <c r="I6" s="7" t="n">
         <v>185.2</v>
       </c>
-      <c r="J6" s="6" t="inlineStr"/>
-      <c r="K6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="4" t="n">
         <v>45844</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>6 Jul</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D7" s="8" t="n">
+      <c r="C7" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D7" s="7" t="n">
         <v>185.4</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="7" t="n">
         <v>240.3</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="7" t="n">
         <v>206.9</v>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="G7" s="7" t="n">
         <v>183.2</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H7" s="7" t="n">
         <v>186.9</v>
       </c>
-      <c r="I7" s="8" t="n">
+      <c r="I7" s="7" t="n">
         <v>185.2</v>
       </c>
-      <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="4" t="n">
         <v>45851</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>13 Jul</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D8" s="8" t="n">
+      <c r="C8" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D8" s="7" t="n">
         <v>184.9</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="7" t="n">
         <v>240.1</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="7" t="n">
         <v>206.6</v>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="7" t="n">
         <v>182</v>
       </c>
-      <c r="H8" s="8" t="n">
+      <c r="H8" s="7" t="n">
         <v>185.7</v>
       </c>
-      <c r="I8" s="8" t="n">
+      <c r="I8" s="7" t="n">
         <v>184</v>
       </c>
-      <c r="J8" s="6" t="inlineStr"/>
-      <c r="K8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="4" t="n">
         <v>45858</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>20 Jul</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D9" s="8" t="n">
+      <c r="C9" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D9" s="7" t="n">
         <v>184.6</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="7" t="n">
         <v>240.2</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="7" t="n">
         <v>206.4</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="7" t="n">
         <v>181.4</v>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="H9" s="7" t="n">
         <v>185.3</v>
       </c>
-      <c r="I9" s="8" t="n">
+      <c r="I9" s="7" t="n">
         <v>183.5</v>
       </c>
-      <c r="J9" s="6" t="inlineStr"/>
-      <c r="K9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="4" t="n">
         <v>45865</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>27 Jul</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D10" s="8" t="n">
+      <c r="C10" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D10" s="7" t="n">
         <v>184.8</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="7" t="n">
         <v>240.6</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="7" t="n">
         <v>206.7</v>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="G10" s="7" t="n">
         <v>181.7</v>
       </c>
-      <c r="H10" s="8" t="n">
+      <c r="H10" s="7" t="n">
         <v>185.5</v>
       </c>
-      <c r="I10" s="8" t="n">
+      <c r="I10" s="7" t="n">
         <v>183.8</v>
       </c>
-      <c r="J10" s="6" t="inlineStr"/>
-      <c r="K10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="4" t="n">
         <v>45872</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>3 Aug</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D11" s="8" t="n">
+      <c r="C11" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D11" s="7" t="n">
         <v>184.9</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="7" t="n">
         <v>240.9</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="7" t="n">
         <v>206.9</v>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="G11" s="7" t="n">
         <v>182</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H11" s="7" t="n">
         <v>185.5</v>
       </c>
-      <c r="I11" s="8" t="n">
+      <c r="I11" s="7" t="n">
         <v>183.9</v>
       </c>
-      <c r="J11" s="6" t="inlineStr"/>
-      <c r="K11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n">
+      <c r="A12" s="4" t="n">
         <v>45879</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>10 Aug</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D12" s="8" t="n">
+      <c r="C12" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D12" s="7" t="n">
         <v>186.2</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="7" t="n">
         <v>241</v>
       </c>
-      <c r="F12" s="8" t="n">
+      <c r="F12" s="7" t="n">
         <v>207.7</v>
       </c>
-      <c r="G12" s="8" t="n">
+      <c r="G12" s="7" t="n">
         <v>184</v>
       </c>
-      <c r="H12" s="8" t="n">
+      <c r="H12" s="7" t="n">
         <v>186.6</v>
       </c>
-      <c r="I12" s="8" t="n">
+      <c r="I12" s="7" t="n">
         <v>185.4</v>
       </c>
-      <c r="J12" s="6" t="inlineStr"/>
-      <c r="K12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n">
+      <c r="A13" s="4" t="n">
         <v>45886</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>17 Aug</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D13" s="8" t="n">
+      <c r="C13" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D13" s="7" t="n">
         <v>186.7</v>
       </c>
-      <c r="E13" s="8" t="n">
+      <c r="E13" s="7" t="n">
         <v>240.8</v>
       </c>
-      <c r="F13" s="8" t="n">
+      <c r="F13" s="7" t="n">
         <v>207.9</v>
       </c>
-      <c r="G13" s="8" t="n">
+      <c r="G13" s="7" t="n">
         <v>184.8</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="H13" s="7" t="n">
         <v>187.2</v>
       </c>
-      <c r="I13" s="8" t="n">
+      <c r="I13" s="7" t="n">
         <v>186.1</v>
       </c>
-      <c r="J13" s="6" t="inlineStr"/>
-      <c r="K13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n">
+      <c r="A14" s="4" t="n">
         <v>45893</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>24 Aug</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D14" s="8" t="n">
+      <c r="C14" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D14" s="7" t="n">
         <v>186.8</v>
       </c>
-      <c r="E14" s="8" t="n">
+      <c r="E14" s="7" t="n">
         <v>240.8</v>
       </c>
-      <c r="F14" s="8" t="n">
+      <c r="F14" s="7" t="n">
         <v>208</v>
       </c>
-      <c r="G14" s="8" t="n">
+      <c r="G14" s="7" t="n">
         <v>183.9</v>
       </c>
-      <c r="H14" s="8" t="n">
+      <c r="H14" s="7" t="n">
         <v>186.8</v>
       </c>
-      <c r="I14" s="8" t="n">
+      <c r="I14" s="7" t="n">
         <v>185.5</v>
       </c>
-      <c r="J14" s="6" t="inlineStr"/>
-      <c r="K14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n">
+      <c r="A15" s="4" t="n">
         <v>45900</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>31 Aug</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D15" s="8" t="n">
+      <c r="C15" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D15" s="7" t="n">
         <v>187.1</v>
       </c>
-      <c r="E15" s="8" t="n">
+      <c r="E15" s="7" t="n">
         <v>241</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="F15" s="7" t="n">
         <v>208.3</v>
       </c>
-      <c r="G15" s="8" t="n">
+      <c r="G15" s="7" t="n">
         <v>183.7</v>
       </c>
-      <c r="H15" s="8" t="n">
+      <c r="H15" s="7" t="n">
         <v>186.6</v>
       </c>
-      <c r="I15" s="8" t="n">
+      <c r="I15" s="7" t="n">
         <v>185.3</v>
       </c>
-      <c r="J15" s="6" t="inlineStr"/>
-      <c r="K15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n">
+      <c r="A16" s="4" t="n">
         <v>45907</v>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>7 Sep</t>
         </is>
       </c>
-      <c r="C16" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D16" s="8" t="n">
+      <c r="C16" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D16" s="7" t="n">
         <v>188.5</v>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="E16" s="7" t="n">
         <v>241.1</v>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="F16" s="7" t="n">
         <v>209.1</v>
       </c>
-      <c r="G16" s="8" t="n">
+      <c r="G16" s="7" t="n">
         <v>184.1</v>
       </c>
-      <c r="H16" s="8" t="n">
+      <c r="H16" s="7" t="n">
         <v>186.9</v>
       </c>
-      <c r="I16" s="8" t="n">
+      <c r="I16" s="7" t="n">
         <v>185.6</v>
       </c>
-      <c r="J16" s="6" t="inlineStr"/>
-      <c r="K16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n">
+      <c r="A17" s="4" t="n">
         <v>45914</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>14 Sep</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D17" s="8" t="n">
+      <c r="C17" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D17" s="7" t="n">
         <v>189.1</v>
       </c>
-      <c r="E17" s="8" t="n">
+      <c r="E17" s="7" t="n">
         <v>241.4</v>
       </c>
-      <c r="F17" s="8" t="n">
+      <c r="F17" s="7" t="n">
         <v>209.6</v>
       </c>
-      <c r="G17" s="8" t="n">
+      <c r="G17" s="7" t="n">
         <v>184.4</v>
       </c>
-      <c r="H17" s="8" t="n">
+      <c r="H17" s="7" t="n">
         <v>187.1</v>
       </c>
-      <c r="I17" s="8" t="n">
+      <c r="I17" s="7" t="n">
         <v>185.9</v>
       </c>
-      <c r="J17" s="6" t="inlineStr"/>
-      <c r="K17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n">
+      <c r="A18" s="4" t="n">
         <v>45921</v>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>21 Sep</t>
         </is>
       </c>
-      <c r="C18" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D18" s="8" t="n">
+      <c r="C18" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D18" s="7" t="n">
         <v>189.2</v>
       </c>
-      <c r="E18" s="8" t="n">
+      <c r="E18" s="7" t="n">
         <v>241.4</v>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="F18" s="7" t="n">
         <v>209.7</v>
       </c>
-      <c r="G18" s="8" t="n">
+      <c r="G18" s="7" t="n">
         <v>184.6</v>
       </c>
-      <c r="H18" s="8" t="n">
+      <c r="H18" s="7" t="n">
         <v>187</v>
       </c>
-      <c r="I18" s="8" t="n">
+      <c r="I18" s="7" t="n">
         <v>185.9</v>
       </c>
-      <c r="J18" s="6" t="inlineStr"/>
-      <c r="K18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="4" t="n">
         <v>45928</v>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>28 Sep</t>
         </is>
       </c>
-      <c r="C19" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D19" s="8" t="n">
+      <c r="C19" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D19" s="7" t="n">
         <v>189.4</v>
       </c>
-      <c r="E19" s="8" t="n">
+      <c r="E19" s="7" t="n">
         <v>241.3</v>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="F19" s="7" t="n">
         <v>209.8</v>
       </c>
-      <c r="G19" s="8" t="n">
+      <c r="G19" s="7" t="n">
         <v>184.3</v>
       </c>
-      <c r="H19" s="8" t="n">
+      <c r="H19" s="7" t="n">
         <v>186.9</v>
       </c>
-      <c r="I19" s="8" t="n">
+      <c r="I19" s="7" t="n">
         <v>185.7</v>
       </c>
-      <c r="J19" s="6" t="inlineStr"/>
-      <c r="K19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n">
+      <c r="A20" s="4" t="n">
         <v>45935</v>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>5 Oct</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D20" s="8" t="n">
+      <c r="C20" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D20" s="7" t="n">
         <v>189.6</v>
       </c>
-      <c r="E20" s="8" t="n">
+      <c r="E20" s="7" t="n">
         <v>241.3</v>
       </c>
-      <c r="F20" s="8" t="n">
+      <c r="F20" s="7" t="n">
         <v>209.9</v>
       </c>
-      <c r="G20" s="8" t="n">
+      <c r="G20" s="7" t="n">
         <v>184</v>
       </c>
-      <c r="H20" s="8" t="n">
+      <c r="H20" s="7" t="n">
         <v>186.9</v>
       </c>
-      <c r="I20" s="8" t="n">
+      <c r="I20" s="7" t="n">
         <v>185.6</v>
       </c>
-      <c r="J20" s="6" t="inlineStr"/>
-      <c r="K20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="n">
+      <c r="A21" s="4" t="n">
         <v>45942</v>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>12 Oct</t>
         </is>
       </c>
-      <c r="C21" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D21" s="8" t="n">
+      <c r="C21" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D21" s="7" t="n">
         <v>189.5</v>
       </c>
-      <c r="E21" s="8" t="n">
+      <c r="E21" s="7" t="n">
         <v>241.4</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="F21" s="7" t="n">
         <v>209.9</v>
       </c>
-      <c r="G21" s="8" t="n">
+      <c r="G21" s="7" t="n">
         <v>184.1</v>
       </c>
-      <c r="H21" s="8" t="n">
+      <c r="H21" s="7" t="n">
         <v>186.9</v>
       </c>
-      <c r="I21" s="8" t="n">
+      <c r="I21" s="7" t="n">
         <v>185.6</v>
       </c>
-      <c r="J21" s="6" t="inlineStr"/>
-      <c r="K21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="n">
+      <c r="A22" s="4" t="n">
         <v>45949</v>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>19 Oct</t>
         </is>
       </c>
-      <c r="C22" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D22" s="8" t="n">
+      <c r="C22" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D22" s="7" t="n">
         <v>189.1</v>
       </c>
-      <c r="E22" s="8" t="n">
+      <c r="E22" s="7" t="n">
         <v>241.4</v>
       </c>
-      <c r="F22" s="8" t="n">
+      <c r="F22" s="7" t="n">
         <v>209.6</v>
       </c>
-      <c r="G22" s="8" t="n">
+      <c r="G22" s="7" t="n">
         <v>183.2</v>
       </c>
-      <c r="H22" s="8" t="n">
+      <c r="H22" s="7" t="n">
         <v>185.9</v>
       </c>
-      <c r="I22" s="8" t="n">
+      <c r="I22" s="7" t="n">
         <v>184.7</v>
       </c>
-      <c r="J22" s="6" t="inlineStr"/>
-      <c r="K22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="n">
+      <c r="A23" s="4" t="n">
         <v>45956</v>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>26 Oct</t>
         </is>
       </c>
-      <c r="C23" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D23" s="8" t="n">
+      <c r="C23" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D23" s="7" t="n">
         <v>188.9</v>
       </c>
-      <c r="E23" s="8" t="n">
+      <c r="E23" s="7" t="n">
         <v>241.4</v>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="F23" s="7" t="n">
         <v>209.5</v>
       </c>
-      <c r="G23" s="8" t="n">
+      <c r="G23" s="7" t="n">
         <v>183</v>
       </c>
-      <c r="H23" s="8" t="n">
+      <c r="H23" s="7" t="n">
         <v>184.9</v>
       </c>
-      <c r="I23" s="8" t="n">
+      <c r="I23" s="7" t="n">
         <v>184</v>
       </c>
-      <c r="J23" s="6" t="inlineStr"/>
-      <c r="K23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n">
+      <c r="A24" s="4" t="n">
         <v>45963</v>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>2 Nov</t>
         </is>
       </c>
-      <c r="C24" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D24" s="8" t="n">
+      <c r="C24" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D24" s="7" t="n">
         <v>188.5</v>
       </c>
-      <c r="E24" s="8" t="n">
+      <c r="E24" s="7" t="n">
         <v>241.3</v>
       </c>
-      <c r="F24" s="8" t="n">
+      <c r="F24" s="7" t="n">
         <v>209.2</v>
       </c>
-      <c r="G24" s="8" t="n">
+      <c r="G24" s="7" t="n">
         <v>184.4</v>
       </c>
-      <c r="H24" s="8" t="n">
+      <c r="H24" s="7" t="n">
         <v>185.4</v>
       </c>
-      <c r="I24" s="8" t="n">
+      <c r="I24" s="7" t="n">
         <v>184.9</v>
       </c>
-      <c r="J24" s="6" t="inlineStr"/>
-      <c r="K24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n">
+      <c r="A25" s="4" t="n">
         <v>45970</v>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>9 Nov</t>
         </is>
       </c>
-      <c r="C25" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D25" s="8" t="n">
+      <c r="C25" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D25" s="7" t="n">
         <v>188.6</v>
       </c>
-      <c r="E25" s="8" t="n">
+      <c r="E25" s="7" t="n">
         <v>241.6</v>
       </c>
-      <c r="F25" s="8" t="n">
+      <c r="F25" s="7" t="n">
         <v>209.4</v>
       </c>
-      <c r="G25" s="8" t="n">
+      <c r="G25" s="7" t="n">
         <v>185.5</v>
       </c>
-      <c r="H25" s="8" t="n">
+      <c r="H25" s="7" t="n">
         <v>186.6</v>
       </c>
-      <c r="I25" s="8" t="n">
+      <c r="I25" s="7" t="n">
         <v>186.1</v>
       </c>
-      <c r="J25" s="6" t="inlineStr"/>
-      <c r="K25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="n">
+      <c r="A26" s="4" t="n">
         <v>45977</v>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>16 Nov</t>
         </is>
       </c>
-      <c r="C26" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D26" s="8" t="n">
+      <c r="C26" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D26" s="7" t="n">
         <v>189.7</v>
       </c>
-      <c r="E26" s="8" t="n">
+      <c r="E26" s="7" t="n">
         <v>242.2</v>
       </c>
-      <c r="F26" s="8" t="n">
+      <c r="F26" s="7" t="n">
         <v>210.3</v>
       </c>
-      <c r="G26" s="8" t="n">
+      <c r="G26" s="7" t="n">
         <v>188.5</v>
       </c>
-      <c r="H26" s="8" t="n">
+      <c r="H26" s="7" t="n">
         <v>188.6</v>
       </c>
-      <c r="I26" s="8" t="n">
+      <c r="I26" s="7" t="n">
         <v>188.6</v>
       </c>
-      <c r="J26" s="6" t="inlineStr"/>
-      <c r="K26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="n">
+      <c r="A27" s="4" t="n">
         <v>45984</v>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>23 Nov</t>
         </is>
       </c>
-      <c r="C27" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D27" s="8" t="n">
+      <c r="C27" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D27" s="7" t="n">
         <v>191.5</v>
       </c>
-      <c r="E27" s="8" t="n">
+      <c r="E27" s="7" t="n">
         <v>242.8</v>
       </c>
-      <c r="F27" s="8" t="n">
+      <c r="F27" s="7" t="n">
         <v>211.6</v>
       </c>
-      <c r="G27" s="8" t="n">
+      <c r="G27" s="7" t="n">
         <v>191.1</v>
       </c>
-      <c r="H27" s="8" t="n">
+      <c r="H27" s="7" t="n">
         <v>190.9</v>
       </c>
-      <c r="I27" s="8" t="n">
+      <c r="I27" s="7" t="n">
         <v>191</v>
       </c>
-      <c r="J27" s="6" t="inlineStr"/>
-      <c r="K27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="n">
+      <c r="A28" s="4" t="n">
         <v>45991</v>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>30 Nov</t>
         </is>
       </c>
-      <c r="C28" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D28" s="8" t="n">
+      <c r="C28" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D28" s="7" t="n">
         <v>192.4</v>
       </c>
-      <c r="E28" s="8" t="n">
+      <c r="E28" s="7" t="n">
         <v>242.9</v>
       </c>
-      <c r="F28" s="8" t="n">
+      <c r="F28" s="7" t="n">
         <v>212.2</v>
       </c>
-      <c r="G28" s="8" t="n">
+      <c r="G28" s="7" t="n">
         <v>192.3</v>
       </c>
-      <c r="H28" s="8" t="n">
+      <c r="H28" s="7" t="n">
         <v>192</v>
       </c>
-      <c r="I28" s="8" t="n">
+      <c r="I28" s="7" t="n">
         <v>192.1</v>
       </c>
-      <c r="J28" s="6" t="inlineStr"/>
-      <c r="K28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="n">
+      <c r="A29" s="4" t="n">
         <v>45998</v>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>7 Dec</t>
         </is>
       </c>
-      <c r="C29" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D29" s="8" t="n">
+      <c r="C29" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D29" s="7" t="n">
         <v>191.4</v>
       </c>
-      <c r="E29" s="8" t="n">
+      <c r="E29" s="7" t="n">
         <v>242.5</v>
       </c>
-      <c r="F29" s="8" t="n">
+      <c r="F29" s="7" t="n">
         <v>211.4</v>
       </c>
-      <c r="G29" s="8" t="n">
+      <c r="G29" s="7" t="n">
         <v>191.9</v>
       </c>
-      <c r="H29" s="8" t="n">
+      <c r="H29" s="7" t="n">
         <v>191.6</v>
       </c>
-      <c r="I29" s="8" t="n">
+      <c r="I29" s="7" t="n">
         <v>191.7</v>
       </c>
-      <c r="J29" s="6" t="inlineStr"/>
-      <c r="K29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="n">
+      <c r="A30" s="4" t="n">
         <v>46005</v>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>14 Dec</t>
         </is>
       </c>
-      <c r="C30" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D30" s="8" t="n">
+      <c r="C30" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D30" s="7" t="n">
         <v>191</v>
       </c>
-      <c r="E30" s="8" t="n">
+      <c r="E30" s="7" t="n">
         <v>241.5</v>
       </c>
-      <c r="F30" s="8" t="n">
+      <c r="F30" s="7" t="n">
         <v>210.8</v>
       </c>
-      <c r="G30" s="8" t="n">
+      <c r="G30" s="7" t="n">
         <v>191.1</v>
       </c>
-      <c r="H30" s="8" t="n">
+      <c r="H30" s="7" t="n">
         <v>190.5</v>
       </c>
-      <c r="I30" s="8" t="n">
+      <c r="I30" s="7" t="n">
         <v>190.8</v>
       </c>
-      <c r="J30" s="6" t="inlineStr"/>
-      <c r="K30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="n">
+      <c r="A31" s="4" t="n">
         <v>46012</v>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>21 Dec</t>
         </is>
       </c>
-      <c r="C31" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D31" s="8" t="n">
+      <c r="C31" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D31" s="7" t="n">
         <v>189.2</v>
       </c>
-      <c r="E31" s="8" t="n">
+      <c r="E31" s="7" t="n">
         <v>240.9</v>
       </c>
-      <c r="F31" s="8" t="n">
+      <c r="F31" s="7" t="n">
         <v>209.5</v>
       </c>
-      <c r="G31" s="8" t="n">
+      <c r="G31" s="7" t="n">
         <v>189.4</v>
       </c>
-      <c r="H31" s="8" t="n">
+      <c r="H31" s="7" t="n">
         <v>189.2</v>
       </c>
-      <c r="I31" s="8" t="n">
+      <c r="I31" s="7" t="n">
         <v>189.3</v>
       </c>
-      <c r="J31" s="6" t="inlineStr"/>
-      <c r="K31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="n">
+      <c r="A32" s="4" t="n">
         <v>46019</v>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>28 Dec</t>
         </is>
       </c>
-      <c r="C32" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D32" s="8" t="n">
+      <c r="C32" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D32" s="7" t="n">
         <v>188</v>
       </c>
-      <c r="E32" s="8" t="n">
+      <c r="E32" s="7" t="n">
         <v>240.5</v>
       </c>
-      <c r="F32" s="8" t="n">
+      <c r="F32" s="7" t="n">
         <v>208.6</v>
       </c>
-      <c r="G32" s="8" t="n">
+      <c r="G32" s="7" t="n">
         <v>187</v>
       </c>
-      <c r="H32" s="8" t="n">
+      <c r="H32" s="7" t="n">
         <v>187.5</v>
       </c>
-      <c r="I32" s="8" t="n">
+      <c r="I32" s="7" t="n">
         <v>187.3</v>
       </c>
-      <c r="J32" s="6" t="inlineStr"/>
-      <c r="K32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="n">
+      <c r="A33" s="4" t="n">
         <v>46026</v>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>4 Jan</t>
         </is>
       </c>
-      <c r="C33" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D33" s="8" t="n">
+      <c r="C33" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D33" s="7" t="n">
         <v>187.5</v>
       </c>
-      <c r="E33" s="8" t="n">
+      <c r="E33" s="7" t="n">
         <v>240.3</v>
       </c>
-      <c r="F33" s="8" t="n">
+      <c r="F33" s="7" t="n">
         <v>208.2</v>
       </c>
-      <c r="G33" s="8" t="n">
+      <c r="G33" s="7" t="n">
         <v>185.6</v>
       </c>
-      <c r="H33" s="8" t="n">
+      <c r="H33" s="7" t="n">
         <v>186.5</v>
       </c>
-      <c r="I33" s="8" t="n">
+      <c r="I33" s="7" t="n">
         <v>186.1</v>
       </c>
-      <c r="J33" s="6" t="inlineStr"/>
-      <c r="K33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="n">
+      <c r="A34" s="4" t="n">
         <v>46033</v>
       </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>11 Jan</t>
         </is>
       </c>
-      <c r="C34" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D34" s="8" t="n">
+      <c r="C34" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D34" s="7" t="n">
         <v>186.3</v>
       </c>
-      <c r="E34" s="8" t="n">
+      <c r="E34" s="7" t="n">
         <v>239.6</v>
       </c>
-      <c r="F34" s="8" t="n">
+      <c r="F34" s="7" t="n">
         <v>207.2</v>
       </c>
-      <c r="G34" s="8" t="n">
+      <c r="G34" s="7" t="n">
         <v>183.6</v>
       </c>
-      <c r="H34" s="8" t="n">
+      <c r="H34" s="7" t="n">
         <v>185.1</v>
       </c>
-      <c r="I34" s="8" t="n">
+      <c r="I34" s="7" t="n">
         <v>184.4</v>
       </c>
-      <c r="J34" s="6" t="inlineStr"/>
-      <c r="K34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="n">
+      <c r="A35" s="4" t="n">
         <v>46040</v>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>18 Jan</t>
         </is>
       </c>
-      <c r="C35" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D35" s="8" t="n">
+      <c r="C35" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D35" s="7" t="n">
         <v>186.1</v>
       </c>
-      <c r="E35" s="8" t="n">
+      <c r="E35" s="7" t="n">
         <v>239.5</v>
       </c>
-      <c r="F35" s="8" t="n">
+      <c r="F35" s="7" t="n">
         <v>207</v>
       </c>
-      <c r="G35" s="8" t="n">
+      <c r="G35" s="7" t="n">
         <v>182.2</v>
       </c>
-      <c r="H35" s="8" t="n">
+      <c r="H35" s="7" t="n">
         <v>183.8</v>
       </c>
-      <c r="I35" s="8" t="n">
+      <c r="I35" s="7" t="n">
         <v>183.1</v>
       </c>
-      <c r="J35" s="6" t="inlineStr"/>
-      <c r="K35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="n">
+      <c r="A36" s="4" t="n">
         <v>46047</v>
       </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>25 Jan</t>
         </is>
       </c>
-      <c r="C36" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D36" s="8" t="n">
+      <c r="C36" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D36" s="7" t="n">
         <v>185.5</v>
       </c>
-      <c r="E36" s="8" t="n">
+      <c r="E36" s="7" t="n">
         <v>239.1</v>
       </c>
-      <c r="F36" s="8" t="n">
+      <c r="F36" s="7" t="n">
         <v>206.5</v>
       </c>
-      <c r="G36" s="8" t="n">
+      <c r="G36" s="7" t="n">
         <v>180.9</v>
       </c>
-      <c r="H36" s="8" t="n">
+      <c r="H36" s="7" t="n">
         <v>183.2</v>
       </c>
-      <c r="I36" s="8" t="n">
+      <c r="I36" s="7" t="n">
         <v>182.1</v>
       </c>
-      <c r="J36" s="6" t="inlineStr"/>
-      <c r="K36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="n">
+      <c r="A37" s="4" t="n">
         <v>46054</v>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>1 Feb</t>
         </is>
       </c>
-      <c r="C37" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D37" s="8" t="n">
+      <c r="C37" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D37" s="7" t="n">
         <v>184.1</v>
       </c>
-      <c r="E37" s="8" t="n">
+      <c r="E37" s="7" t="n">
         <v>238.6</v>
       </c>
-      <c r="F37" s="8" t="n">
+      <c r="F37" s="7" t="n">
         <v>205.5</v>
       </c>
-      <c r="G37" s="8" t="n">
+      <c r="G37" s="7" t="n">
         <v>179.9</v>
       </c>
-      <c r="H37" s="8" t="n">
+      <c r="H37" s="7" t="n">
         <v>182.7</v>
       </c>
-      <c r="I37" s="8" t="n">
+      <c r="I37" s="7" t="n">
         <v>181.4</v>
       </c>
-      <c r="J37" s="6" t="inlineStr"/>
-      <c r="K37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="n">
+      <c r="A38" s="4" t="n">
         <v>46061</v>
       </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>8 Feb</t>
         </is>
       </c>
-      <c r="C38" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D38" s="8" t="n">
+      <c r="C38" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D38" s="7" t="n">
         <v>183.1</v>
       </c>
-      <c r="E38" s="8" t="n">
+      <c r="E38" s="7" t="n">
         <v>238</v>
       </c>
-      <c r="F38" s="8" t="n">
+      <c r="F38" s="7" t="n">
         <v>204.7</v>
       </c>
-      <c r="G38" s="8" t="n">
+      <c r="G38" s="7" t="n">
         <v>179.1</v>
       </c>
-      <c r="H38" s="8" t="n">
+      <c r="H38" s="7" t="n">
         <v>182.2</v>
       </c>
-      <c r="I38" s="8" t="n">
+      <c r="I38" s="7" t="n">
         <v>180.8</v>
       </c>
-      <c r="J38" s="6" t="inlineStr"/>
-      <c r="K38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="n">
+      <c r="A39" s="4" t="n">
         <v>46068</v>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>15 Feb</t>
         </is>
       </c>
-      <c r="C39" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D39" s="8" t="n">
+      <c r="C39" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D39" s="7" t="n">
         <v>182.6</v>
       </c>
-      <c r="E39" s="8" t="n">
+      <c r="E39" s="7" t="n">
         <v>237.9</v>
       </c>
-      <c r="F39" s="8" t="n">
+      <c r="F39" s="7" t="n">
         <v>204.3</v>
       </c>
-      <c r="G39" s="8" t="n">
+      <c r="G39" s="7" t="n">
         <v>178.6</v>
       </c>
-      <c r="H39" s="8" t="n">
+      <c r="H39" s="7" t="n">
         <v>182</v>
       </c>
-      <c r="I39" s="8" t="n">
+      <c r="I39" s="7" t="n">
         <v>180.5</v>
       </c>
-      <c r="J39" s="6" t="inlineStr"/>
-      <c r="K39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="n">
+      <c r="A40" s="4" t="n">
         <v>46075</v>
       </c>
-      <c r="B40" s="6" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>22 Feb</t>
         </is>
       </c>
-      <c r="C40" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D40" s="8" t="n">
+      <c r="C40" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D40" s="7" t="n">
         <v>182.5</v>
       </c>
-      <c r="E40" s="8" t="n">
+      <c r="E40" s="7" t="n">
         <v>237.9</v>
       </c>
-      <c r="F40" s="8" t="n">
+      <c r="F40" s="7" t="n">
         <v>204.2</v>
       </c>
-      <c r="G40" s="8" t="n">
+      <c r="G40" s="7" t="n">
         <v>178.2</v>
       </c>
-      <c r="H40" s="8" t="n">
+      <c r="H40" s="7" t="n">
         <v>181.8</v>
       </c>
-      <c r="I40" s="8" t="n">
+      <c r="I40" s="7" t="n">
         <v>180.2</v>
       </c>
-      <c r="J40" s="6" t="inlineStr"/>
-      <c r="K40" s="6" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="n">
+      <c r="A41" s="4" t="n">
         <v>46082</v>
       </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>1 Mar</t>
         </is>
       </c>
-      <c r="C41" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D41" s="8" t="n">
+      <c r="C41" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D41" s="7" t="n">
         <v>183.6</v>
       </c>
-      <c r="E41" s="8" t="n">
+      <c r="E41" s="7" t="n">
         <v>237.9</v>
       </c>
-      <c r="F41" s="8" t="n">
+      <c r="F41" s="7" t="n">
         <v>204.9</v>
       </c>
-      <c r="G41" s="8" t="n">
+      <c r="G41" s="7" t="n">
         <v>179.3</v>
       </c>
-      <c r="H41" s="8" t="n">
+      <c r="H41" s="7" t="n">
         <v>182.3</v>
       </c>
-      <c r="I41" s="8" t="n">
+      <c r="I41" s="7" t="n">
         <v>180.9</v>
       </c>
-      <c r="J41" s="6" t="inlineStr"/>
-      <c r="K41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="n">
+      <c r="A42" s="4" t="n">
         <v>46089</v>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>8 Mar</t>
         </is>
       </c>
-      <c r="C42" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D42" s="8" t="n">
+      <c r="C42" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D42" s="7" t="n">
         <v>199.5</v>
       </c>
-      <c r="E42" s="8" t="n">
+      <c r="E42" s="7" t="n">
         <v>242.9</v>
       </c>
-      <c r="F42" s="8" t="n">
+      <c r="F42" s="7" t="n">
         <v>216.5</v>
       </c>
-      <c r="G42" s="8" t="n">
+      <c r="G42" s="7" t="n">
         <v>196.2</v>
       </c>
-      <c r="H42" s="8" t="n">
+      <c r="H42" s="7" t="n">
         <v>196.8</v>
       </c>
-      <c r="I42" s="8" t="n">
+      <c r="I42" s="7" t="n">
         <v>196.5</v>
       </c>
-      <c r="J42" s="6" t="inlineStr"/>
-      <c r="K42" s="6" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="n">
+      <c r="A43" s="4" t="n">
         <v>46096</v>
       </c>
-      <c r="B43" s="6" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>15 Mar</t>
         </is>
       </c>
-      <c r="C43" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D43" s="8" t="n">
+      <c r="C43" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D43" s="7" t="n">
         <v>247</v>
       </c>
-      <c r="E43" s="8" t="n">
+      <c r="E43" s="7" t="n">
         <v>264.3</v>
       </c>
-      <c r="F43" s="8" t="n">
+      <c r="F43" s="7" t="n">
         <v>253.8</v>
       </c>
-      <c r="G43" s="8" t="n">
+      <c r="G43" s="7" t="n">
         <v>245.4</v>
       </c>
-      <c r="H43" s="8" t="n">
+      <c r="H43" s="7" t="n">
         <v>245.8</v>
       </c>
-      <c r="I43" s="8" t="n">
+      <c r="I43" s="7" t="n">
         <v>245.6</v>
       </c>
-      <c r="J43" s="6" t="inlineStr"/>
-      <c r="K43" s="6" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="n">
+      <c r="A44" s="4" t="n">
         <v>46103</v>
       </c>
-      <c r="B44" s="6" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>22 Mar</t>
         </is>
       </c>
-      <c r="C44" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D44" s="8" t="n">
+      <c r="C44" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D44" s="7" t="n">
         <v>281.6</v>
       </c>
-      <c r="E44" s="8" t="n">
+      <c r="E44" s="7" t="n">
         <v>286.5</v>
       </c>
-      <c r="F44" s="8" t="n">
+      <c r="F44" s="7" t="n">
         <v>283.5</v>
       </c>
-      <c r="G44" s="8" t="n">
+      <c r="G44" s="7" t="n">
         <v>281.4</v>
       </c>
-      <c r="H44" s="8" t="n">
+      <c r="H44" s="7" t="n">
         <v>283.2</v>
       </c>
-      <c r="I44" s="8" t="n">
+      <c r="I44" s="7" t="n">
         <v>282.4</v>
       </c>
-      <c r="J44" s="6" t="inlineStr"/>
-      <c r="K44" s="6" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="n">
+      <c r="A45" s="4" t="n">
         <v>46110</v>
       </c>
-      <c r="B45" s="6" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>29 Mar</t>
         </is>
       </c>
-      <c r="C45" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D45" s="8" t="n">
+      <c r="C45" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D45" s="7" t="n">
         <v>308</v>
       </c>
-      <c r="E45" s="8" t="n">
+      <c r="E45" s="7" t="n">
         <v>305</v>
       </c>
-      <c r="F45" s="8" t="n">
+      <c r="F45" s="7" t="n">
         <v>306.8</v>
       </c>
-      <c r="G45" s="8" t="n">
+      <c r="G45" s="7" t="n">
         <v>308.7</v>
       </c>
-      <c r="H45" s="8" t="n">
+      <c r="H45" s="7" t="n">
         <v>311.1</v>
       </c>
-      <c r="I45" s="8" t="n">
+      <c r="I45" s="7" t="n">
         <v>310</v>
       </c>
-      <c r="J45" s="6" t="inlineStr"/>
-      <c r="K45" s="6" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="n">
+      <c r="A46" s="4" t="n">
         <v>46117</v>
       </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>5 Apr</t>
         </is>
       </c>
-      <c r="C46" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D46" s="8" t="n">
+      <c r="C46" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D46" s="7" t="n">
         <v>309.5</v>
       </c>
-      <c r="E46" s="8" t="n">
+      <c r="E46" s="7" t="n">
         <v>317.2</v>
       </c>
-      <c r="F46" s="8" t="n">
+      <c r="F46" s="7" t="n">
         <v>312.5</v>
       </c>
-      <c r="G46" s="8" t="n">
+      <c r="G46" s="7" t="n">
         <v>310.3</v>
       </c>
-      <c r="H46" s="8" t="n">
+      <c r="H46" s="7" t="n">
         <v>314.6</v>
       </c>
-      <c r="I46" s="8" t="n">
+      <c r="I46" s="7" t="n">
         <v>312.7</v>
       </c>
-      <c r="J46" s="6" t="inlineStr"/>
-      <c r="K46" s="6" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="n">
+      <c r="A47" s="4" t="n">
         <v>46124</v>
       </c>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>12 Apr</t>
         </is>
       </c>
-      <c r="C47" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D47" s="8" t="n">
+      <c r="C47" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D47" s="7" t="n">
         <v>319.3</v>
       </c>
-      <c r="E47" s="8" t="n">
+      <c r="E47" s="7" t="n">
         <v>327</v>
       </c>
-      <c r="F47" s="8" t="n">
+      <c r="F47" s="7" t="n">
         <v>322.3</v>
       </c>
-      <c r="G47" s="8" t="n">
+      <c r="G47" s="7" t="n">
         <v>317.1</v>
       </c>
-      <c r="H47" s="8" t="n">
+      <c r="H47" s="7" t="n">
         <v>320.5</v>
       </c>
-      <c r="I47" s="8" t="n">
+      <c r="I47" s="7" t="n">
         <v>319</v>
       </c>
-      <c r="J47" s="6" t="inlineStr"/>
-      <c r="K47" s="6" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="n">
+      <c r="A48" s="4" t="n">
         <v>46131</v>
       </c>
-      <c r="B48" s="6" t="inlineStr">
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>19 Apr</t>
         </is>
       </c>
-      <c r="C48" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D48" s="8" t="n">
+      <c r="C48" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D48" s="7" t="n">
         <v>305.6</v>
       </c>
-      <c r="E48" s="8" t="n">
+      <c r="E48" s="7" t="n">
         <v>325.5</v>
       </c>
-      <c r="F48" s="8" t="n">
+      <c r="F48" s="7" t="n">
         <v>313.4</v>
       </c>
-      <c r="G48" s="8" t="n">
+      <c r="G48" s="7" t="n">
         <v>305.3</v>
       </c>
-      <c r="H48" s="8" t="n">
+      <c r="H48" s="7" t="n">
         <v>311.8</v>
       </c>
-      <c r="I48" s="8" t="n">
+      <c r="I48" s="7" t="n">
         <v>308.9</v>
       </c>
-      <c r="J48" s="6" t="inlineStr"/>
-      <c r="K48" s="6" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="n">
+      <c r="A49" s="4" t="n">
         <v>46138</v>
       </c>
-      <c r="B49" s="6" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>26 Apr</t>
         </is>
       </c>
-      <c r="C49" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D49" s="8" t="n">
+      <c r="C49" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D49" s="7" t="n">
         <v>274.6</v>
       </c>
-      <c r="E49" s="8" t="n">
+      <c r="E49" s="7" t="n">
         <v>290.9</v>
       </c>
-      <c r="F49" s="8" t="n">
+      <c r="F49" s="7" t="n">
         <v>281</v>
       </c>
-      <c r="G49" s="8" t="n">
+      <c r="G49" s="7" t="n">
         <v>270</v>
       </c>
-      <c r="H49" s="8" t="n">
+      <c r="H49" s="7" t="n">
         <v>279.1</v>
       </c>
-      <c r="I49" s="8" t="n">
+      <c r="I49" s="7" t="n">
         <v>275</v>
       </c>
-      <c r="J49" s="6" t="inlineStr"/>
-      <c r="K49" s="6" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="n">
+      <c r="A50" s="4" t="n">
         <v>46145</v>
       </c>
-      <c r="B50" s="6" t="inlineStr">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>3 May</t>
         </is>
       </c>
-      <c r="C50" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D50" s="8" t="n">
+      <c r="C50" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D50" s="7" t="n">
         <v>253.4</v>
       </c>
-      <c r="E50" s="8" t="n">
+      <c r="E50" s="7" t="n">
         <v>308.5</v>
       </c>
-      <c r="F50" s="8" t="n">
+      <c r="F50" s="7" t="n">
         <v>275</v>
       </c>
-      <c r="G50" s="8" t="n">
+      <c r="G50" s="7" t="n">
         <v>249.5</v>
       </c>
-      <c r="H50" s="8" t="n">
+      <c r="H50" s="7" t="n">
         <v>258.3</v>
       </c>
-      <c r="I50" s="8" t="n">
+      <c r="I50" s="7" t="n">
         <v>254.3</v>
       </c>
-      <c r="J50" s="6" t="inlineStr"/>
-      <c r="K50" s="6" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="n">
+      <c r="A51" s="4" t="n">
         <v>46152</v>
       </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>10 May</t>
         </is>
       </c>
-      <c r="C51" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D51" s="8" t="n">
+      <c r="C51" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D51" s="7" t="n">
         <v>247.7</v>
       </c>
-      <c r="E51" s="8" t="n">
+      <c r="E51" s="7" t="n">
         <v>303.5</v>
       </c>
-      <c r="F51" s="8" t="n">
+      <c r="F51" s="7" t="n">
         <v>269.6</v>
       </c>
-      <c r="G51" s="8" t="n">
+      <c r="G51" s="7" t="n">
         <v>243</v>
       </c>
-      <c r="H51" s="8" t="n">
+      <c r="H51" s="7" t="n">
         <v>250.6</v>
       </c>
-      <c r="I51" s="8" t="n">
+      <c r="I51" s="7" t="n">
         <v>247.2</v>
       </c>
-      <c r="J51" s="6" t="inlineStr"/>
-      <c r="K51" s="6" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="n">
+      <c r="A52" s="4" t="n">
         <v>46159</v>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>17 May</t>
         </is>
       </c>
-      <c r="C52" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D52" s="8" t="n">
+      <c r="C52" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D52" s="7" t="n">
         <v>240.8</v>
       </c>
-      <c r="E52" s="8" t="n">
+      <c r="E52" s="7" t="n">
         <v>300.5</v>
       </c>
-      <c r="F52" s="8" t="n">
+      <c r="F52" s="7" t="n">
         <v>264.2</v>
       </c>
-      <c r="G52" s="8" t="n">
+      <c r="G52" s="7" t="n">
         <v>233.2</v>
       </c>
-      <c r="H52" s="8" t="n">
+      <c r="H52" s="7" t="n">
         <v>239.5</v>
       </c>
-      <c r="I52" s="8" t="n">
+      <c r="I52" s="7" t="n">
         <v>236.6</v>
       </c>
-      <c r="J52" s="6" t="inlineStr"/>
-      <c r="K52" s="6" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="n">
+      <c r="A53" s="4" t="n">
         <v>46166</v>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>24 May</t>
         </is>
       </c>
-      <c r="C53" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D53" s="8" t="n">
+      <c r="C53" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="7" t="n">
         <v>236.2</v>
       </c>
-      <c r="E53" s="8" t="n">
+      <c r="E53" s="7" t="n">
         <v>296.5</v>
       </c>
-      <c r="F53" s="8" t="n">
+      <c r="F53" s="7" t="n">
         <v>259.9</v>
       </c>
-      <c r="G53" s="8" t="n">
+      <c r="G53" s="7" t="n">
         <v>227.7</v>
       </c>
-      <c r="H53" s="8" t="n">
+      <c r="H53" s="7" t="n">
         <v>233</v>
       </c>
-      <c r="I53" s="8" t="n">
+      <c r="I53" s="7" t="n">
         <v>230.6</v>
       </c>
-      <c r="J53" s="6" t="inlineStr"/>
-      <c r="K53" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K53"/>
+  <autoFilter ref="A1:I53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2278,7 +2152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2290,8 +2164,6 @@
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2340,1739 +2212,1621 @@
           <t>National Average</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>Excise Cut (1 Apr)</t>
-        </is>
-      </c>
-      <c r="K1" s="4" t="inlineStr">
-        <is>
-          <t>Fuel Price Lock (20 Apr)</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n">
+      <c r="A2" s="4" t="n">
         <v>45809</v>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>1 Jun</t>
         </is>
       </c>
-      <c r="C2" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D2" s="8" t="n">
+      <c r="C2" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D2" s="7" t="n">
         <v>177.7</v>
       </c>
-      <c r="E2" s="8" t="n">
+      <c r="E2" s="7" t="n">
         <v>233.1</v>
       </c>
-      <c r="F2" s="8" t="n">
+      <c r="F2" s="7" t="n">
         <v>192.6</v>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="G2" s="7" t="n">
         <v>178</v>
       </c>
-      <c r="H2" s="8" t="n">
+      <c r="H2" s="7" t="n">
         <v>173.2</v>
       </c>
-      <c r="I2" s="8" t="n">
+      <c r="I2" s="7" t="n">
         <v>176.4</v>
       </c>
-      <c r="J2" s="8" t="n">
-        <v>300</v>
-      </c>
-      <c r="K2" s="8" t="n">
-        <v>300</v>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="4" t="n">
         <v>45816</v>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>8 Jun</t>
         </is>
       </c>
-      <c r="C3" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D3" s="8" t="n">
+      <c r="C3" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D3" s="7" t="n">
         <v>176.9</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="7" t="n">
         <v>232.4</v>
       </c>
-      <c r="F3" s="8" t="n">
+      <c r="F3" s="7" t="n">
         <v>191.8</v>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="G3" s="7" t="n">
         <v>183.3</v>
       </c>
-      <c r="H3" s="8" t="n">
+      <c r="H3" s="7" t="n">
         <v>175.3</v>
       </c>
-      <c r="I3" s="8" t="n">
+      <c r="I3" s="7" t="n">
         <v>180.7</v>
       </c>
-      <c r="J3" s="6" t="inlineStr"/>
-      <c r="K3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="4" t="n">
         <v>45823</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>15 Jun</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D4" s="8" t="n">
+      <c r="C4" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D4" s="7" t="n">
         <v>176.4</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="7" t="n">
         <v>231.5</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="7" t="n">
         <v>191.2</v>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="G4" s="7" t="n">
         <v>180.6</v>
       </c>
-      <c r="H4" s="8" t="n">
+      <c r="H4" s="7" t="n">
         <v>174.4</v>
       </c>
-      <c r="I4" s="8" t="n">
+      <c r="I4" s="7" t="n">
         <v>178.6</v>
       </c>
-      <c r="J4" s="6" t="inlineStr"/>
-      <c r="K4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="4" t="n">
         <v>45830</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>22 Jun</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D5" s="8" t="n">
+      <c r="C5" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D5" s="7" t="n">
         <v>177.8</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="7" t="n">
         <v>231.5</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="7" t="n">
         <v>192.2</v>
       </c>
-      <c r="G5" s="8" t="n">
+      <c r="G5" s="7" t="n">
         <v>174.2</v>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="H5" s="7" t="n">
         <v>176.5</v>
       </c>
-      <c r="I5" s="8" t="n">
+      <c r="I5" s="7" t="n">
         <v>175</v>
       </c>
-      <c r="J5" s="6" t="inlineStr"/>
-      <c r="K5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="4" t="n">
         <v>45837</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>29 Jun</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D6" s="8" t="n">
+      <c r="C6" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D6" s="7" t="n">
         <v>180.7</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="7" t="n">
         <v>232.2</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="7" t="n">
         <v>194.6</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="7" t="n">
         <v>178.5</v>
       </c>
-      <c r="H6" s="8" t="n">
+      <c r="H6" s="7" t="n">
         <v>179.7</v>
       </c>
-      <c r="I6" s="8" t="n">
+      <c r="I6" s="7" t="n">
         <v>178.9</v>
       </c>
-      <c r="J6" s="6" t="inlineStr"/>
-      <c r="K6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="4" t="n">
         <v>45844</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>6 Jul</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D7" s="8" t="n">
+      <c r="C7" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D7" s="7" t="n">
         <v>181.4</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="7" t="n">
         <v>232.2</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="7" t="n">
         <v>195.1</v>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="G7" s="7" t="n">
         <v>186.3</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H7" s="7" t="n">
         <v>179.6</v>
       </c>
-      <c r="I7" s="8" t="n">
+      <c r="I7" s="7" t="n">
         <v>184</v>
       </c>
-      <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="4" t="n">
         <v>45851</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>13 Jul</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D8" s="8" t="n">
+      <c r="C8" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D8" s="7" t="n">
         <v>181.1</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="7" t="n">
         <v>232</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="7" t="n">
         <v>194.8</v>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="7" t="n">
         <v>188.9</v>
       </c>
-      <c r="H8" s="8" t="n">
+      <c r="H8" s="7" t="n">
         <v>178.8</v>
       </c>
-      <c r="I8" s="8" t="n">
+      <c r="I8" s="7" t="n">
         <v>185.6</v>
       </c>
-      <c r="J8" s="6" t="inlineStr"/>
-      <c r="K8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="4" t="n">
         <v>45858</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>20 Jul</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D9" s="8" t="n">
+      <c r="C9" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D9" s="7" t="n">
         <v>179.8</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="7" t="n">
         <v>231.9</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="7" t="n">
         <v>193.8</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="7" t="n">
         <v>177.6</v>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="H9" s="7" t="n">
         <v>177.2</v>
       </c>
-      <c r="I9" s="8" t="n">
+      <c r="I9" s="7" t="n">
         <v>177.5</v>
       </c>
-      <c r="J9" s="6" t="inlineStr"/>
-      <c r="K9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="4" t="n">
         <v>45865</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>27 Jul</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D10" s="8" t="n">
+      <c r="C10" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D10" s="7" t="n">
         <v>179.4</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="7" t="n">
         <v>232.3</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="7" t="n">
         <v>193.6</v>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="G10" s="7" t="n">
         <v>171</v>
       </c>
-      <c r="H10" s="8" t="n">
+      <c r="H10" s="7" t="n">
         <v>176</v>
       </c>
-      <c r="I10" s="8" t="n">
+      <c r="I10" s="7" t="n">
         <v>172.6</v>
       </c>
-      <c r="J10" s="6" t="inlineStr"/>
-      <c r="K10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="4" t="n">
         <v>45872</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>3 Aug</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D11" s="8" t="n">
+      <c r="C11" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D11" s="7" t="n">
         <v>179.7</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="7" t="n">
         <v>233</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="7" t="n">
         <v>194</v>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="G11" s="7" t="n">
         <v>168.6</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H11" s="7" t="n">
         <v>175.3</v>
       </c>
-      <c r="I11" s="8" t="n">
+      <c r="I11" s="7" t="n">
         <v>170.8</v>
       </c>
-      <c r="J11" s="6" t="inlineStr"/>
-      <c r="K11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n">
+      <c r="A12" s="4" t="n">
         <v>45879</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>10 Aug</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D12" s="8" t="n">
+      <c r="C12" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D12" s="7" t="n">
         <v>181.2</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="7" t="n">
         <v>233.9</v>
       </c>
-      <c r="F12" s="8" t="n">
+      <c r="F12" s="7" t="n">
         <v>195.4</v>
       </c>
-      <c r="G12" s="8" t="n">
+      <c r="G12" s="7" t="n">
         <v>179.6</v>
       </c>
-      <c r="H12" s="8" t="n">
+      <c r="H12" s="7" t="n">
         <v>176.1</v>
       </c>
-      <c r="I12" s="8" t="n">
+      <c r="I12" s="7" t="n">
         <v>178.5</v>
       </c>
-      <c r="J12" s="6" t="inlineStr"/>
-      <c r="K12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n">
+      <c r="A13" s="4" t="n">
         <v>45886</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>17 Aug</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D13" s="8" t="n">
+      <c r="C13" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D13" s="7" t="n">
         <v>182.2</v>
       </c>
-      <c r="E13" s="8" t="n">
+      <c r="E13" s="7" t="n">
         <v>234.2</v>
       </c>
-      <c r="F13" s="8" t="n">
+      <c r="F13" s="7" t="n">
         <v>196.2</v>
       </c>
-      <c r="G13" s="8" t="n">
+      <c r="G13" s="7" t="n">
         <v>185.4</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="H13" s="7" t="n">
         <v>176.8</v>
       </c>
-      <c r="I13" s="8" t="n">
+      <c r="I13" s="7" t="n">
         <v>182.6</v>
       </c>
-      <c r="J13" s="6" t="inlineStr"/>
-      <c r="K13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n">
+      <c r="A14" s="4" t="n">
         <v>45893</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>24 Aug</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D14" s="8" t="n">
+      <c r="C14" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D14" s="7" t="n">
         <v>182.8</v>
       </c>
-      <c r="E14" s="8" t="n">
+      <c r="E14" s="7" t="n">
         <v>234.3</v>
       </c>
-      <c r="F14" s="8" t="n">
+      <c r="F14" s="7" t="n">
         <v>196.6</v>
       </c>
-      <c r="G14" s="8" t="n">
+      <c r="G14" s="7" t="n">
         <v>181.8</v>
       </c>
-      <c r="H14" s="8" t="n">
+      <c r="H14" s="7" t="n">
         <v>176.6</v>
       </c>
-      <c r="I14" s="8" t="n">
+      <c r="I14" s="7" t="n">
         <v>180.1</v>
       </c>
-      <c r="J14" s="6" t="inlineStr"/>
-      <c r="K14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n">
+      <c r="A15" s="4" t="n">
         <v>45900</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>31 Aug</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D15" s="8" t="n">
+      <c r="C15" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D15" s="7" t="n">
         <v>184</v>
       </c>
-      <c r="E15" s="8" t="n">
+      <c r="E15" s="7" t="n">
         <v>234.7</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="F15" s="7" t="n">
         <v>197.6</v>
       </c>
-      <c r="G15" s="8" t="n">
+      <c r="G15" s="7" t="n">
         <v>175.7</v>
       </c>
-      <c r="H15" s="8" t="n">
+      <c r="H15" s="7" t="n">
         <v>176.8</v>
       </c>
-      <c r="I15" s="8" t="n">
+      <c r="I15" s="7" t="n">
         <v>176</v>
       </c>
-      <c r="J15" s="6" t="inlineStr"/>
-      <c r="K15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n">
+      <c r="A16" s="4" t="n">
         <v>45907</v>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>7 Sep</t>
         </is>
       </c>
-      <c r="C16" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D16" s="8" t="n">
+      <c r="C16" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D16" s="7" t="n">
         <v>186</v>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="E16" s="7" t="n">
         <v>235.1</v>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="F16" s="7" t="n">
         <v>199.2</v>
       </c>
-      <c r="G16" s="8" t="n">
+      <c r="G16" s="7" t="n">
         <v>175.2</v>
       </c>
-      <c r="H16" s="8" t="n">
+      <c r="H16" s="7" t="n">
         <v>177.4</v>
       </c>
-      <c r="I16" s="8" t="n">
+      <c r="I16" s="7" t="n">
         <v>175.9</v>
       </c>
-      <c r="J16" s="6" t="inlineStr"/>
-      <c r="K16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n">
+      <c r="A17" s="4" t="n">
         <v>45914</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>14 Sep</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D17" s="8" t="n">
+      <c r="C17" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D17" s="7" t="n">
         <v>187</v>
       </c>
-      <c r="E17" s="8" t="n">
+      <c r="E17" s="7" t="n">
         <v>235.5</v>
       </c>
-      <c r="F17" s="8" t="n">
+      <c r="F17" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="G17" s="8" t="n">
+      <c r="G17" s="7" t="n">
         <v>180.4</v>
       </c>
-      <c r="H17" s="8" t="n">
+      <c r="H17" s="7" t="n">
         <v>177.8</v>
       </c>
-      <c r="I17" s="8" t="n">
+      <c r="I17" s="7" t="n">
         <v>179.5</v>
       </c>
-      <c r="J17" s="6" t="inlineStr"/>
-      <c r="K17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n">
+      <c r="A18" s="4" t="n">
         <v>45921</v>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>21 Sep</t>
         </is>
       </c>
-      <c r="C18" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D18" s="8" t="n">
+      <c r="C18" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D18" s="7" t="n">
         <v>187.3</v>
       </c>
-      <c r="E18" s="8" t="n">
+      <c r="E18" s="7" t="n">
         <v>235.7</v>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="F18" s="7" t="n">
         <v>200.3</v>
       </c>
-      <c r="G18" s="8" t="n">
+      <c r="G18" s="7" t="n">
         <v>187.4</v>
       </c>
-      <c r="H18" s="8" t="n">
+      <c r="H18" s="7" t="n">
         <v>178.2</v>
       </c>
-      <c r="I18" s="8" t="n">
+      <c r="I18" s="7" t="n">
         <v>184.4</v>
       </c>
-      <c r="J18" s="6" t="inlineStr"/>
-      <c r="K18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="4" t="n">
         <v>45928</v>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>28 Sep</t>
         </is>
       </c>
-      <c r="C19" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D19" s="8" t="n">
+      <c r="C19" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D19" s="7" t="n">
         <v>187</v>
       </c>
-      <c r="E19" s="8" t="n">
+      <c r="E19" s="7" t="n">
         <v>236</v>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="F19" s="7" t="n">
         <v>200.2</v>
       </c>
-      <c r="G19" s="8" t="n">
+      <c r="G19" s="7" t="n">
         <v>188.1</v>
       </c>
-      <c r="H19" s="8" t="n">
+      <c r="H19" s="7" t="n">
         <v>178.4</v>
       </c>
-      <c r="I19" s="8" t="n">
+      <c r="I19" s="7" t="n">
         <v>184.9</v>
       </c>
-      <c r="J19" s="6" t="inlineStr"/>
-      <c r="K19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n">
+      <c r="A20" s="4" t="n">
         <v>45935</v>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>5 Oct</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D20" s="8" t="n">
+      <c r="C20" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D20" s="7" t="n">
         <v>186.8</v>
       </c>
-      <c r="E20" s="8" t="n">
+      <c r="E20" s="7" t="n">
         <v>236</v>
       </c>
-      <c r="F20" s="8" t="n">
+      <c r="F20" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="G20" s="8" t="n">
+      <c r="G20" s="7" t="n">
         <v>179.6</v>
       </c>
-      <c r="H20" s="8" t="n">
+      <c r="H20" s="7" t="n">
         <v>177.9</v>
       </c>
-      <c r="I20" s="8" t="n">
+      <c r="I20" s="7" t="n">
         <v>179.1</v>
       </c>
-      <c r="J20" s="6" t="inlineStr"/>
-      <c r="K20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="n">
+      <c r="A21" s="4" t="n">
         <v>45942</v>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>12 Oct</t>
         </is>
       </c>
-      <c r="C21" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D21" s="8" t="n">
+      <c r="C21" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D21" s="7" t="n">
         <v>187</v>
       </c>
-      <c r="E21" s="8" t="n">
+      <c r="E21" s="7" t="n">
         <v>236</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="F21" s="7" t="n">
         <v>200.2</v>
       </c>
-      <c r="G21" s="8" t="n">
+      <c r="G21" s="7" t="n">
         <v>176.2</v>
       </c>
-      <c r="H21" s="8" t="n">
+      <c r="H21" s="7" t="n">
         <v>177.4</v>
       </c>
-      <c r="I21" s="8" t="n">
+      <c r="I21" s="7" t="n">
         <v>176.6</v>
       </c>
-      <c r="J21" s="6" t="inlineStr"/>
-      <c r="K21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="n">
+      <c r="A22" s="4" t="n">
         <v>45949</v>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>19 Oct</t>
         </is>
       </c>
-      <c r="C22" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D22" s="8" t="n">
+      <c r="C22" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D22" s="7" t="n">
         <v>187.1</v>
       </c>
-      <c r="E22" s="8" t="n">
+      <c r="E22" s="7" t="n">
         <v>236.1</v>
       </c>
-      <c r="F22" s="8" t="n">
+      <c r="F22" s="7" t="n">
         <v>200.2</v>
       </c>
-      <c r="G22" s="8" t="n">
+      <c r="G22" s="7" t="n">
         <v>176.5</v>
       </c>
-      <c r="H22" s="8" t="n">
+      <c r="H22" s="7" t="n">
         <v>176.5</v>
       </c>
-      <c r="I22" s="8" t="n">
+      <c r="I22" s="7" t="n">
         <v>176.5</v>
       </c>
-      <c r="J22" s="6" t="inlineStr"/>
-      <c r="K22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="n">
+      <c r="A23" s="4" t="n">
         <v>45956</v>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>26 Oct</t>
         </is>
       </c>
-      <c r="C23" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D23" s="8" t="n">
+      <c r="C23" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D23" s="7" t="n">
         <v>186.9</v>
       </c>
-      <c r="E23" s="8" t="n">
+      <c r="E23" s="7" t="n">
         <v>235.6</v>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="F23" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="G23" s="8" t="n">
+      <c r="G23" s="7" t="n">
         <v>182.2</v>
       </c>
-      <c r="H23" s="8" t="n">
+      <c r="H23" s="7" t="n">
         <v>176.3</v>
       </c>
-      <c r="I23" s="8" t="n">
+      <c r="I23" s="7" t="n">
         <v>180.2</v>
       </c>
-      <c r="J23" s="6" t="inlineStr"/>
-      <c r="K23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n">
+      <c r="A24" s="4" t="n">
         <v>45963</v>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>2 Nov</t>
         </is>
       </c>
-      <c r="C24" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D24" s="8" t="n">
+      <c r="C24" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D24" s="7" t="n">
         <v>187.1</v>
       </c>
-      <c r="E24" s="8" t="n">
+      <c r="E24" s="7" t="n">
         <v>235.5</v>
       </c>
-      <c r="F24" s="8" t="n">
+      <c r="F24" s="7" t="n">
         <v>200.1</v>
       </c>
-      <c r="G24" s="8" t="n">
+      <c r="G24" s="7" t="n">
         <v>187.4</v>
       </c>
-      <c r="H24" s="8" t="n">
+      <c r="H24" s="7" t="n">
         <v>177.2</v>
       </c>
-      <c r="I24" s="8" t="n">
+      <c r="I24" s="7" t="n">
         <v>184.1</v>
       </c>
-      <c r="J24" s="6" t="inlineStr"/>
-      <c r="K24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n">
+      <c r="A25" s="4" t="n">
         <v>45970</v>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>9 Nov</t>
         </is>
       </c>
-      <c r="C25" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D25" s="8" t="n">
+      <c r="C25" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D25" s="7" t="n">
         <v>187.6</v>
       </c>
-      <c r="E25" s="8" t="n">
+      <c r="E25" s="7" t="n">
         <v>236.4</v>
       </c>
-      <c r="F25" s="8" t="n">
+      <c r="F25" s="7" t="n">
         <v>200.7</v>
       </c>
-      <c r="G25" s="8" t="n">
+      <c r="G25" s="7" t="n">
         <v>184.3</v>
       </c>
-      <c r="H25" s="8" t="n">
+      <c r="H25" s="7" t="n">
         <v>177.5</v>
       </c>
-      <c r="I25" s="8" t="n">
+      <c r="I25" s="7" t="n">
         <v>182.1</v>
       </c>
-      <c r="J25" s="6" t="inlineStr"/>
-      <c r="K25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="n">
+      <c r="A26" s="4" t="n">
         <v>45977</v>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>16 Nov</t>
         </is>
       </c>
-      <c r="C26" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D26" s="8" t="n">
+      <c r="C26" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D26" s="7" t="n">
         <v>187.8</v>
       </c>
-      <c r="E26" s="8" t="n">
+      <c r="E26" s="7" t="n">
         <v>236.5</v>
       </c>
-      <c r="F26" s="8" t="n">
+      <c r="F26" s="7" t="n">
         <v>200.9</v>
       </c>
-      <c r="G26" s="8" t="n">
+      <c r="G26" s="7" t="n">
         <v>181.5</v>
       </c>
-      <c r="H26" s="8" t="n">
+      <c r="H26" s="7" t="n">
         <v>177.7</v>
       </c>
-      <c r="I26" s="8" t="n">
+      <c r="I26" s="7" t="n">
         <v>180.3</v>
       </c>
-      <c r="J26" s="6" t="inlineStr"/>
-      <c r="K26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="n">
+      <c r="A27" s="4" t="n">
         <v>45984</v>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>23 Nov</t>
         </is>
       </c>
-      <c r="C27" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D27" s="8" t="n">
+      <c r="C27" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D27" s="7" t="n">
         <v>187.9</v>
       </c>
-      <c r="E27" s="8" t="n">
+      <c r="E27" s="7" t="n">
         <v>235.9</v>
       </c>
-      <c r="F27" s="8" t="n">
+      <c r="F27" s="7" t="n">
         <v>200.8</v>
       </c>
-      <c r="G27" s="8" t="n">
+      <c r="G27" s="7" t="n">
         <v>183.4</v>
       </c>
-      <c r="H27" s="8" t="n">
+      <c r="H27" s="7" t="n">
         <v>178.1</v>
       </c>
-      <c r="I27" s="8" t="n">
+      <c r="I27" s="7" t="n">
         <v>181.6</v>
       </c>
-      <c r="J27" s="6" t="inlineStr"/>
-      <c r="K27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="n">
+      <c r="A28" s="4" t="n">
         <v>45991</v>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>30 Nov</t>
         </is>
       </c>
-      <c r="C28" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D28" s="8" t="n">
+      <c r="C28" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D28" s="7" t="n">
         <v>187.8</v>
       </c>
-      <c r="E28" s="8" t="n">
+      <c r="E28" s="7" t="n">
         <v>235.8</v>
       </c>
-      <c r="F28" s="8" t="n">
+      <c r="F28" s="7" t="n">
         <v>200.7</v>
       </c>
-      <c r="G28" s="8" t="n">
+      <c r="G28" s="7" t="n">
         <v>187.8</v>
       </c>
-      <c r="H28" s="8" t="n">
+      <c r="H28" s="7" t="n">
         <v>178.5</v>
       </c>
-      <c r="I28" s="8" t="n">
+      <c r="I28" s="7" t="n">
         <v>184.7</v>
       </c>
-      <c r="J28" s="6" t="inlineStr"/>
-      <c r="K28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="n">
+      <c r="A29" s="4" t="n">
         <v>45998</v>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>7 Dec</t>
         </is>
       </c>
-      <c r="C29" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D29" s="8" t="n">
+      <c r="C29" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D29" s="7" t="n">
         <v>187.1</v>
       </c>
-      <c r="E29" s="8" t="n">
+      <c r="E29" s="7" t="n">
         <v>235.5</v>
       </c>
-      <c r="F29" s="8" t="n">
+      <c r="F29" s="7" t="n">
         <v>200.1</v>
       </c>
-      <c r="G29" s="8" t="n">
+      <c r="G29" s="7" t="n">
         <v>189.8</v>
       </c>
-      <c r="H29" s="8" t="n">
+      <c r="H29" s="7" t="n">
         <v>178.7</v>
       </c>
-      <c r="I29" s="8" t="n">
+      <c r="I29" s="7" t="n">
         <v>186.1</v>
       </c>
-      <c r="J29" s="6" t="inlineStr"/>
-      <c r="K29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="n">
+      <c r="A30" s="4" t="n">
         <v>46005</v>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>14 Dec</t>
         </is>
       </c>
-      <c r="C30" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D30" s="8" t="n">
+      <c r="C30" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D30" s="7" t="n">
         <v>185.9</v>
       </c>
-      <c r="E30" s="8" t="n">
+      <c r="E30" s="7" t="n">
         <v>234.7</v>
       </c>
-      <c r="F30" s="8" t="n">
+      <c r="F30" s="7" t="n">
         <v>199</v>
       </c>
-      <c r="G30" s="8" t="n">
+      <c r="G30" s="7" t="n">
         <v>189.7</v>
       </c>
-      <c r="H30" s="8" t="n">
+      <c r="H30" s="7" t="n">
         <v>178.2</v>
       </c>
-      <c r="I30" s="8" t="n">
+      <c r="I30" s="7" t="n">
         <v>185.9</v>
       </c>
-      <c r="J30" s="6" t="inlineStr"/>
-      <c r="K30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="n">
+      <c r="A31" s="4" t="n">
         <v>46012</v>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>21 Dec</t>
         </is>
       </c>
-      <c r="C31" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D31" s="8" t="n">
+      <c r="C31" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D31" s="7" t="n">
         <v>184.5</v>
       </c>
-      <c r="E31" s="8" t="n">
+      <c r="E31" s="7" t="n">
         <v>234.4</v>
       </c>
-      <c r="F31" s="8" t="n">
+      <c r="F31" s="7" t="n">
         <v>197.9</v>
       </c>
-      <c r="G31" s="8" t="n">
+      <c r="G31" s="7" t="n">
         <v>181.2</v>
       </c>
-      <c r="H31" s="8" t="n">
+      <c r="H31" s="7" t="n">
         <v>176.8</v>
       </c>
-      <c r="I31" s="8" t="n">
+      <c r="I31" s="7" t="n">
         <v>179.8</v>
       </c>
-      <c r="J31" s="6" t="inlineStr"/>
-      <c r="K31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="n">
+      <c r="A32" s="4" t="n">
         <v>46019</v>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>28 Dec</t>
         </is>
       </c>
-      <c r="C32" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D32" s="8" t="n">
+      <c r="C32" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D32" s="7" t="n">
         <v>184.1</v>
       </c>
-      <c r="E32" s="8" t="n">
+      <c r="E32" s="7" t="n">
         <v>234.3</v>
       </c>
-      <c r="F32" s="8" t="n">
+      <c r="F32" s="7" t="n">
         <v>197.6</v>
       </c>
-      <c r="G32" s="8" t="n">
+      <c r="G32" s="7" t="n">
         <v>175.1</v>
       </c>
-      <c r="H32" s="8" t="n">
+      <c r="H32" s="7" t="n">
         <v>175.3</v>
       </c>
-      <c r="I32" s="8" t="n">
+      <c r="I32" s="7" t="n">
         <v>175.2</v>
       </c>
-      <c r="J32" s="6" t="inlineStr"/>
-      <c r="K32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="n">
+      <c r="A33" s="4" t="n">
         <v>46026</v>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>4 Jan</t>
         </is>
       </c>
-      <c r="C33" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D33" s="8" t="n">
+      <c r="C33" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D33" s="7" t="n">
         <v>184</v>
       </c>
-      <c r="E33" s="8" t="n">
+      <c r="E33" s="7" t="n">
         <v>234.4</v>
       </c>
-      <c r="F33" s="8" t="n">
+      <c r="F33" s="7" t="n">
         <v>197.6</v>
       </c>
-      <c r="G33" s="8" t="n">
+      <c r="G33" s="7" t="n">
         <v>176</v>
       </c>
-      <c r="H33" s="8" t="n">
+      <c r="H33" s="7" t="n">
         <v>174.7</v>
       </c>
-      <c r="I33" s="8" t="n">
+      <c r="I33" s="7" t="n">
         <v>175.6</v>
       </c>
-      <c r="J33" s="6" t="inlineStr"/>
-      <c r="K33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="n">
+      <c r="A34" s="4" t="n">
         <v>46033</v>
       </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>11 Jan</t>
         </is>
       </c>
-      <c r="C34" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D34" s="8" t="n">
+      <c r="C34" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D34" s="7" t="n">
         <v>183.8</v>
       </c>
-      <c r="E34" s="8" t="n">
+      <c r="E34" s="7" t="n">
         <v>234.3</v>
       </c>
-      <c r="F34" s="8" t="n">
+      <c r="F34" s="7" t="n">
         <v>197.4</v>
       </c>
-      <c r="G34" s="8" t="n">
+      <c r="G34" s="7" t="n">
         <v>180.4</v>
       </c>
-      <c r="H34" s="8" t="n">
+      <c r="H34" s="7" t="n">
         <v>174.2</v>
       </c>
-      <c r="I34" s="8" t="n">
+      <c r="I34" s="7" t="n">
         <v>178.3</v>
       </c>
-      <c r="J34" s="6" t="inlineStr"/>
-      <c r="K34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="n">
+      <c r="A35" s="4" t="n">
         <v>46040</v>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>18 Jan</t>
         </is>
       </c>
-      <c r="C35" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D35" s="8" t="n">
+      <c r="C35" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D35" s="7" t="n">
         <v>183.7</v>
       </c>
-      <c r="E35" s="8" t="n">
+      <c r="E35" s="7" t="n">
         <v>234.1</v>
       </c>
-      <c r="F35" s="8" t="n">
+      <c r="F35" s="7" t="n">
         <v>197.3</v>
       </c>
-      <c r="G35" s="8" t="n">
+      <c r="G35" s="7" t="n">
         <v>182.2</v>
       </c>
-      <c r="H35" s="8" t="n">
+      <c r="H35" s="7" t="n">
         <v>173.4</v>
       </c>
-      <c r="I35" s="8" t="n">
+      <c r="I35" s="7" t="n">
         <v>179.3</v>
       </c>
-      <c r="J35" s="6" t="inlineStr"/>
-      <c r="K35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="n">
+      <c r="A36" s="4" t="n">
         <v>46047</v>
       </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>25 Jan</t>
         </is>
       </c>
-      <c r="C36" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D36" s="8" t="n">
+      <c r="C36" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D36" s="7" t="n">
         <v>182.8</v>
       </c>
-      <c r="E36" s="8" t="n">
+      <c r="E36" s="7" t="n">
         <v>233.8</v>
       </c>
-      <c r="F36" s="8" t="n">
+      <c r="F36" s="7" t="n">
         <v>196.5</v>
       </c>
-      <c r="G36" s="8" t="n">
+      <c r="G36" s="7" t="n">
         <v>178.5</v>
       </c>
-      <c r="H36" s="8" t="n">
+      <c r="H36" s="7" t="n">
         <v>172.5</v>
       </c>
-      <c r="I36" s="8" t="n">
+      <c r="I36" s="7" t="n">
         <v>176.5</v>
       </c>
-      <c r="J36" s="6" t="inlineStr"/>
-      <c r="K36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="n">
+      <c r="A37" s="4" t="n">
         <v>46054</v>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>1 Feb</t>
         </is>
       </c>
-      <c r="C37" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D37" s="8" t="n">
+      <c r="C37" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D37" s="7" t="n">
         <v>181.4</v>
       </c>
-      <c r="E37" s="8" t="n">
+      <c r="E37" s="7" t="n">
         <v>232.9</v>
       </c>
-      <c r="F37" s="8" t="n">
+      <c r="F37" s="7" t="n">
         <v>195.2</v>
       </c>
-      <c r="G37" s="8" t="n">
+      <c r="G37" s="7" t="n">
         <v>170.3</v>
       </c>
-      <c r="H37" s="8" t="n">
+      <c r="H37" s="7" t="n">
         <v>171.6</v>
       </c>
-      <c r="I37" s="8" t="n">
+      <c r="I37" s="7" t="n">
         <v>170.7</v>
       </c>
-      <c r="J37" s="6" t="inlineStr"/>
-      <c r="K37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="n">
+      <c r="A38" s="4" t="n">
         <v>46061</v>
       </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>8 Feb</t>
         </is>
       </c>
-      <c r="C38" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D38" s="8" t="n">
+      <c r="C38" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D38" s="7" t="n">
         <v>180.1</v>
       </c>
-      <c r="E38" s="8" t="n">
+      <c r="E38" s="7" t="n">
         <v>231.8</v>
       </c>
-      <c r="F38" s="8" t="n">
+      <c r="F38" s="7" t="n">
         <v>194</v>
       </c>
-      <c r="G38" s="8" t="n">
+      <c r="G38" s="7" t="n">
         <v>163.8</v>
       </c>
-      <c r="H38" s="8" t="n">
+      <c r="H38" s="7" t="n">
         <v>170.8</v>
       </c>
-      <c r="I38" s="8" t="n">
+      <c r="I38" s="7" t="n">
         <v>166.1</v>
       </c>
-      <c r="J38" s="6" t="inlineStr"/>
-      <c r="K38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="n">
+      <c r="A39" s="4" t="n">
         <v>46068</v>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>15 Feb</t>
         </is>
       </c>
-      <c r="C39" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D39" s="8" t="n">
+      <c r="C39" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D39" s="7" t="n">
         <v>179.2</v>
       </c>
-      <c r="E39" s="8" t="n">
+      <c r="E39" s="7" t="n">
         <v>231.7</v>
       </c>
-      <c r="F39" s="8" t="n">
+      <c r="F39" s="7" t="n">
         <v>193.3</v>
       </c>
-      <c r="G39" s="8" t="n">
+      <c r="G39" s="7" t="n">
         <v>164.8</v>
       </c>
-      <c r="H39" s="8" t="n">
+      <c r="H39" s="7" t="n">
         <v>170.1</v>
       </c>
-      <c r="I39" s="8" t="n">
+      <c r="I39" s="7" t="n">
         <v>166.6</v>
       </c>
-      <c r="J39" s="6" t="inlineStr"/>
-      <c r="K39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="n">
+      <c r="A40" s="4" t="n">
         <v>46075</v>
       </c>
-      <c r="B40" s="6" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>22 Feb</t>
         </is>
       </c>
-      <c r="C40" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D40" s="8" t="n">
+      <c r="C40" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D40" s="7" t="n">
         <v>179.1</v>
       </c>
-      <c r="E40" s="8" t="n">
+      <c r="E40" s="7" t="n">
         <v>232.3</v>
       </c>
-      <c r="F40" s="8" t="n">
+      <c r="F40" s="7" t="n">
         <v>193.4</v>
       </c>
-      <c r="G40" s="8" t="n">
+      <c r="G40" s="7" t="n">
         <v>171.7</v>
       </c>
-      <c r="H40" s="8" t="n">
+      <c r="H40" s="7" t="n">
         <v>169.6</v>
       </c>
-      <c r="I40" s="8" t="n">
+      <c r="I40" s="7" t="n">
         <v>171</v>
       </c>
-      <c r="J40" s="6" t="inlineStr"/>
-      <c r="K40" s="6" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="n">
+      <c r="A41" s="4" t="n">
         <v>46082</v>
       </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>1 Mar</t>
         </is>
       </c>
-      <c r="C41" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D41" s="8" t="n">
+      <c r="C41" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D41" s="7" t="n">
         <v>179.4</v>
       </c>
-      <c r="E41" s="8" t="n">
+      <c r="E41" s="7" t="n">
         <v>232.4</v>
       </c>
-      <c r="F41" s="8" t="n">
+      <c r="F41" s="7" t="n">
         <v>193.6</v>
       </c>
-      <c r="G41" s="8" t="n">
+      <c r="G41" s="7" t="n">
         <v>186.4</v>
       </c>
-      <c r="H41" s="8" t="n">
+      <c r="H41" s="7" t="n">
         <v>170.1</v>
       </c>
-      <c r="I41" s="8" t="n">
+      <c r="I41" s="7" t="n">
         <v>181</v>
       </c>
-      <c r="J41" s="6" t="inlineStr"/>
-      <c r="K41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="n">
+      <c r="A42" s="4" t="n">
         <v>46089</v>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>8 Mar</t>
         </is>
       </c>
-      <c r="C42" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D42" s="8" t="n">
+      <c r="C42" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D42" s="7" t="n">
         <v>193.6</v>
       </c>
-      <c r="E42" s="8" t="n">
+      <c r="E42" s="7" t="n">
         <v>234.9</v>
       </c>
-      <c r="F42" s="8" t="n">
+      <c r="F42" s="7" t="n">
         <v>204.7</v>
       </c>
-      <c r="G42" s="8" t="n">
+      <c r="G42" s="7" t="n">
         <v>203.5</v>
       </c>
-      <c r="H42" s="8" t="n">
+      <c r="H42" s="7" t="n">
         <v>186.7</v>
       </c>
-      <c r="I42" s="8" t="n">
+      <c r="I42" s="7" t="n">
         <v>198</v>
       </c>
-      <c r="J42" s="6" t="inlineStr"/>
-      <c r="K42" s="6" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="n">
+      <c r="A43" s="4" t="n">
         <v>46096</v>
       </c>
-      <c r="B43" s="6" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>15 Mar</t>
         </is>
       </c>
-      <c r="C43" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D43" s="8" t="n">
+      <c r="C43" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D43" s="7" t="n">
         <v>227.1</v>
       </c>
-      <c r="E43" s="8" t="n">
+      <c r="E43" s="7" t="n">
         <v>248.8</v>
       </c>
-      <c r="F43" s="8" t="n">
+      <c r="F43" s="7" t="n">
         <v>232.9</v>
       </c>
-      <c r="G43" s="8" t="n">
+      <c r="G43" s="7" t="n">
         <v>220.4</v>
       </c>
-      <c r="H43" s="8" t="n">
+      <c r="H43" s="7" t="n">
         <v>217.6</v>
       </c>
-      <c r="I43" s="8" t="n">
+      <c r="I43" s="7" t="n">
         <v>219.5</v>
       </c>
-      <c r="J43" s="6" t="inlineStr"/>
-      <c r="K43" s="6" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="n">
+      <c r="A44" s="4" t="n">
         <v>46103</v>
       </c>
-      <c r="B44" s="6" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>22 Mar</t>
         </is>
       </c>
-      <c r="C44" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D44" s="8" t="n">
+      <c r="C44" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D44" s="7" t="n">
         <v>243.5</v>
       </c>
-      <c r="E44" s="8" t="n">
+      <c r="E44" s="7" t="n">
         <v>263.9</v>
       </c>
-      <c r="F44" s="8" t="n">
+      <c r="F44" s="7" t="n">
         <v>249</v>
       </c>
-      <c r="G44" s="8" t="n">
+      <c r="G44" s="7" t="n">
         <v>237.2</v>
       </c>
-      <c r="H44" s="8" t="n">
+      <c r="H44" s="7" t="n">
         <v>239.6</v>
       </c>
-      <c r="I44" s="8" t="n">
+      <c r="I44" s="7" t="n">
         <v>238</v>
       </c>
-      <c r="J44" s="6" t="inlineStr"/>
-      <c r="K44" s="6" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="n">
+      <c r="A45" s="4" t="n">
         <v>46110</v>
       </c>
-      <c r="B45" s="6" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>29 Mar</t>
         </is>
       </c>
-      <c r="C45" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D45" s="8" t="n">
+      <c r="C45" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D45" s="7" t="n">
         <v>258.5</v>
       </c>
-      <c r="E45" s="8" t="n">
+      <c r="E45" s="7" t="n">
         <v>277</v>
       </c>
-      <c r="F45" s="8" t="n">
+      <c r="F45" s="7" t="n">
         <v>263.5</v>
       </c>
-      <c r="G45" s="8" t="n">
+      <c r="G45" s="7" t="n">
         <v>252.6</v>
       </c>
-      <c r="H45" s="8" t="n">
+      <c r="H45" s="7" t="n">
         <v>255.2</v>
       </c>
-      <c r="I45" s="8" t="n">
+      <c r="I45" s="7" t="n">
         <v>253.4</v>
       </c>
-      <c r="J45" s="6" t="inlineStr"/>
-      <c r="K45" s="6" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="n">
+      <c r="A46" s="4" t="n">
         <v>46117</v>
       </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>5 Apr</t>
         </is>
       </c>
-      <c r="C46" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D46" s="8" t="n">
+      <c r="C46" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D46" s="7" t="n">
         <v>242.3</v>
       </c>
-      <c r="E46" s="8" t="n">
+      <c r="E46" s="7" t="n">
         <v>281.6</v>
       </c>
-      <c r="F46" s="8" t="n">
+      <c r="F46" s="7" t="n">
         <v>252.8</v>
       </c>
-      <c r="G46" s="8" t="n">
+      <c r="G46" s="7" t="n">
         <v>238.9</v>
       </c>
-      <c r="H46" s="8" t="n">
+      <c r="H46" s="7" t="n">
         <v>242.6</v>
       </c>
-      <c r="I46" s="8" t="n">
+      <c r="I46" s="7" t="n">
         <v>240.1</v>
       </c>
-      <c r="J46" s="6" t="inlineStr"/>
-      <c r="K46" s="6" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="n">
+      <c r="A47" s="4" t="n">
         <v>46124</v>
       </c>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>12 Apr</t>
         </is>
       </c>
-      <c r="C47" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D47" s="8" t="n">
+      <c r="C47" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D47" s="7" t="n">
         <v>227.3</v>
       </c>
-      <c r="E47" s="8" t="n">
+      <c r="E47" s="7" t="n">
         <v>283.2</v>
       </c>
-      <c r="F47" s="8" t="n">
+      <c r="F47" s="7" t="n">
         <v>242.3</v>
       </c>
-      <c r="G47" s="8" t="n">
+      <c r="G47" s="7" t="n">
         <v>223</v>
       </c>
-      <c r="H47" s="8" t="n">
+      <c r="H47" s="7" t="n">
         <v>227.4</v>
       </c>
-      <c r="I47" s="8" t="n">
+      <c r="I47" s="7" t="n">
         <v>224.5</v>
       </c>
-      <c r="J47" s="6" t="inlineStr"/>
-      <c r="K47" s="6" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="n">
+      <c r="A48" s="4" t="n">
         <v>46131</v>
       </c>
-      <c r="B48" s="6" t="inlineStr">
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>19 Apr</t>
         </is>
       </c>
-      <c r="C48" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D48" s="8" t="n">
+      <c r="C48" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D48" s="7" t="n">
         <v>215.2</v>
       </c>
-      <c r="E48" s="8" t="n">
+      <c r="E48" s="7" t="n">
         <v>280.7</v>
       </c>
-      <c r="F48" s="8" t="n">
+      <c r="F48" s="7" t="n">
         <v>232.8</v>
       </c>
-      <c r="G48" s="8" t="n">
+      <c r="G48" s="7" t="n">
         <v>211.2</v>
       </c>
-      <c r="H48" s="8" t="n">
+      <c r="H48" s="7" t="n">
         <v>216.4</v>
       </c>
-      <c r="I48" s="8" t="n">
+      <c r="I48" s="7" t="n">
         <v>212.9</v>
       </c>
-      <c r="J48" s="6" t="inlineStr"/>
-      <c r="K48" s="6" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="n">
+      <c r="A49" s="4" t="n">
         <v>46138</v>
       </c>
-      <c r="B49" s="6" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>26 Apr</t>
         </is>
       </c>
-      <c r="C49" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D49" s="8" t="n">
+      <c r="C49" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D49" s="7" t="n">
         <v>198.6</v>
       </c>
-      <c r="E49" s="8" t="n">
+      <c r="E49" s="7" t="n">
         <v>234.6</v>
       </c>
-      <c r="F49" s="8" t="n">
+      <c r="F49" s="7" t="n">
         <v>208.3</v>
       </c>
-      <c r="G49" s="8" t="n">
+      <c r="G49" s="7" t="n">
         <v>189.7</v>
       </c>
-      <c r="H49" s="8" t="n">
+      <c r="H49" s="7" t="n">
         <v>197.5</v>
       </c>
-      <c r="I49" s="8" t="n">
+      <c r="I49" s="7" t="n">
         <v>192.3</v>
       </c>
-      <c r="J49" s="6" t="inlineStr"/>
-      <c r="K49" s="6" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="n">
+      <c r="A50" s="4" t="n">
         <v>46145</v>
       </c>
-      <c r="B50" s="6" t="inlineStr">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>3 May</t>
         </is>
       </c>
-      <c r="C50" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D50" s="8" t="n">
+      <c r="C50" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D50" s="7" t="n">
         <v>193.8</v>
       </c>
-      <c r="E50" s="8" t="n">
+      <c r="E50" s="7" t="n">
         <v>272.1</v>
       </c>
-      <c r="F50" s="8" t="n">
+      <c r="F50" s="7" t="n">
         <v>214.8</v>
       </c>
-      <c r="G50" s="8" t="n">
+      <c r="G50" s="7" t="n">
         <v>180.9</v>
       </c>
-      <c r="H50" s="8" t="n">
+      <c r="H50" s="7" t="n">
         <v>188.7</v>
       </c>
-      <c r="I50" s="8" t="n">
+      <c r="I50" s="7" t="n">
         <v>183.4</v>
       </c>
-      <c r="J50" s="6" t="inlineStr"/>
-      <c r="K50" s="6" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="n">
+      <c r="A51" s="4" t="n">
         <v>46152</v>
       </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>10 May</t>
         </is>
       </c>
-      <c r="C51" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D51" s="8" t="n">
+      <c r="C51" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D51" s="7" t="n">
         <v>192.6</v>
       </c>
-      <c r="E51" s="8" t="n">
+      <c r="E51" s="7" t="n">
         <v>275.3</v>
       </c>
-      <c r="F51" s="8" t="n">
+      <c r="F51" s="7" t="n">
         <v>214.8</v>
       </c>
-      <c r="G51" s="8" t="n">
+      <c r="G51" s="7" t="n">
         <v>181.7</v>
       </c>
-      <c r="H51" s="8" t="n">
+      <c r="H51" s="7" t="n">
         <v>187.5</v>
       </c>
-      <c r="I51" s="8" t="n">
+      <c r="I51" s="7" t="n">
         <v>183.6</v>
       </c>
-      <c r="J51" s="6" t="inlineStr"/>
-      <c r="K51" s="6" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="n">
+      <c r="A52" s="4" t="n">
         <v>46159</v>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>17 May</t>
         </is>
       </c>
-      <c r="C52" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D52" s="8" t="n">
+      <c r="C52" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D52" s="7" t="n">
         <v>191.1</v>
       </c>
-      <c r="E52" s="8" t="n">
+      <c r="E52" s="7" t="n">
         <v>275.6</v>
       </c>
-      <c r="F52" s="8" t="n">
+      <c r="F52" s="7" t="n">
         <v>213.8</v>
       </c>
-      <c r="G52" s="8" t="n">
+      <c r="G52" s="7" t="n">
         <v>183.7</v>
       </c>
-      <c r="H52" s="8" t="n">
+      <c r="H52" s="7" t="n">
         <v>185.4</v>
       </c>
-      <c r="I52" s="8" t="n">
+      <c r="I52" s="7" t="n">
         <v>184.2</v>
       </c>
-      <c r="J52" s="6" t="inlineStr"/>
-      <c r="K52" s="6" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="n">
+      <c r="A53" s="4" t="n">
         <v>46166</v>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>24 May</t>
         </is>
       </c>
-      <c r="C53" s="7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D53" s="8" t="n">
+      <c r="C53" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="7" t="n">
         <v>192.3</v>
       </c>
-      <c r="E53" s="8" t="n">
+      <c r="E53" s="7" t="n">
         <v>269</v>
       </c>
-      <c r="F53" s="8" t="n">
+      <c r="F53" s="7" t="n">
         <v>212.9</v>
       </c>
-      <c r="G53" s="8" t="n">
+      <c r="G53" s="7" t="n">
         <v>185.6</v>
       </c>
-      <c r="H53" s="8" t="n">
+      <c r="H53" s="7" t="n">
         <v>186.4</v>
       </c>
-      <c r="I53" s="8" t="n">
+      <c r="I53" s="7" t="n">
         <v>185.8</v>
       </c>
-      <c r="J53" s="6" t="inlineStr"/>
-      <c r="K53" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K53"/>
+  <autoFilter ref="A1:I53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>